<commit_message>
Update results: Reclassify ANH-028 (deferred tax) from No to Review per §274 Wahlrecht
</commit_message>
<xml_diff>
--- a/output/results.xlsx
+++ b/output/results.xlsx
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -569,7 +569,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
@@ -580,7 +580,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>92.2%</t>
+          <t>94.0%</t>
         </is>
       </c>
     </row>
@@ -695,17 +695,17 @@
         <v>12</v>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n">
         <v>13</v>
       </c>
       <c r="F17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
@@ -3837,19 +3837,19 @@
           <t>Only if the entity has made a policy choice regarding deferred tax recognition</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Review</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>No deferred tax assets or liabilities are recognised on the balance sheet, and the Anhang's accounting policies section does not address deferred taxes (latente Steuern) at all. § 274 HGB requires recognition of deferred tax liabilities for temporary differences; deferred tax assets may be waived under § 274 Abs. 1 S. 2. Whether the entity has waived deferred tax recognition or determined that no material temporary differences exist, the policy choice must be disclosed per § 284 Abs. 2 Nr. 3 HGB. This disclosure is entirely absent.</t>
+          <t>Material temporary differences exist (pensions, BilMoG, discount rate), but no deferred tax assets/liabilities recognised. Under §274 Abs. 1 HGB, recognition is optional for standalone financial statements.</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Cross-references ANH-003 (same gap). Temporary differences from pensions (PUC method, BilMoG amounts, discount rate difference) likely exist but their deferred tax treatment is not discussed.</t>
+          <t>Reclassified from No to Review — recognition is a Wahlrecht under §274 HGB. Need to verify if the entity explicitly elected not to recognise.</t>
         </is>
       </c>
     </row>
@@ -5435,19 +5435,19 @@
           <t>Has the entity disclosed the treatment of aktive latente Steuern (deferred tax assets) and the reasons for any waiver of recognition per § 274 HGB?</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Review</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>No deferred tax assets or liabilities are recognised on the balance sheet, and the Anhang's accounting policies section does not address deferred taxes (latente Steuern) at all. § 274 HGB requires recognition of deferred tax liabilities for temporary differences; deferred tax assets may be waived under § 274 Abs. 1 S. 2. Whether the entity has waived deferred tax recognition or determined that no material temporary differences exist, the policy choice must be disclosed per § 284 Abs. 2 Nr. 3 HGB. This disclosure is entirely absent.</t>
+          <t>Material temporary differences exist (pensions, BilMoG, discount rate), but no deferred tax assets/liabilities recognised. Under §274 Abs. 1 HGB, recognition is optional for standalone financial statements.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Cross-references ANH-003 (same gap). Temporary differences from pensions (PUC method, BilMoG amounts, discount rate difference) likely exist but their deferred tax treatment is not discussed.</t>
+          <t>Reclassified from No to Review — recognition is a Wahlrecht under §274 HGB. Need to verify if the entity explicitly elected not to recognise.</t>
         </is>
       </c>
     </row>

</xml_diff>